<commit_message>
feat(demo): expand samples with compatibility examples
Add DOCX font inheritance, PPTX numbering and preset shape pages, and XLSX palette and tint comparisons to the existing generated samples. Preserve the original content and document where to find each example.

Tested: 14 focused Rust tests, workspace all-target Clippy, rustfmt, deterministic sample generation, packaged asset equality, on-device demo sample navigation and XLSX checks, independent source and visual review
</commit_message>
<xml_diff>
--- a/demo/src/main/assets/samples/sample.xlsx
+++ b/demo/src/main/assets/samples/sample.xlsx
@@ -30,7 +30,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color rgb="FF202124"/>
@@ -42,8 +42,16 @@
       <u/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -60,8 +68,28 @@
         <fgColor rgb="FFE4F0F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0000FF" tint="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0000FF" tint="0.5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0000FF" tint="-0.5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border/>
     <border>
       <left style="thin">
@@ -77,11 +105,25 @@
         <color rgb="FF112233"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="2"/>
+      </left>
+      <top style="thin">
+        <color indexed="2"/>
+      </top>
+      <right style="thin">
+        <color indexed="2"/>
+      </right>
+      <bottom style="thin">
+        <color indexed="2"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -97,7 +139,26 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="2" fillId="4" borderId="2">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="5">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="6">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="7">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00202080"/>
+      <rgbColor rgb="00A0E0C0"/>
+      <rgbColor rgb="00800040"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -160,11 +221,95 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">调色板与明暗色｜B 实际 · C 预期</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">自定义调色板
+字体 / 填充 / 边框</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Palette 调色板</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">深蓝字 · 浅绿底
+四边为紫红色</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">蓝色原色
+tint = 0</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">原色 Blue</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#0000FF
+作为明暗比较基准</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">提高明度
+tint = +0.5</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">变亮 Lighter</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#8080FF
+蓝色变浅，接近白色</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">降低明度
+tint = -0.5</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">变暗 Darker</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#000080
+蓝色变深，接近黑色</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A7:C7"/>
   </mergeCells>
 </worksheet>
 </file>

</xml_diff>